<commit_message>
fix: Se hicieron ajustes para la plantilla y s agrego el tsconfig.json para evitar problemas de compatibilidad
</commit_message>
<xml_diff>
--- a/docs/plantilla-importacion-datos.xlsx
+++ b/docs/plantilla-importacion-datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Desktop\coodetrans-gestion\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B09F3B74-EB3D-423E-BA6A-FF76D9A7442D}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDC4CF45-DD6E-4C64-A440-88182D0A84BC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B9CF0795-0054-4CD1-8B64-60E772BEE863}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{B9CF0795-0054-4CD1-8B64-60E772BEE863}"/>
   </bookViews>
   <sheets>
     <sheet name="Plantilla para Activos" sheetId="1" r:id="rId1"/>
@@ -24,12 +24,7 @@
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
         <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
         <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
       </xcalcf:calcFeatures>
     </ext>
     <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
@@ -40,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="13">
   <si>
     <t>Codigo</t>
   </si>
@@ -73,13 +68,99 @@
   </si>
   <si>
     <t>Esta seria una plantilla para poder hacer una importacion masiva en la base de datos en Retirados</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">La columna </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Novedad</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> da a entender el estado del empleado en general Activo para esta plantilla</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">En </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>F/Novedad</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> sigue el formato MM DD/AAAA (AGO 21/2026) y </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Fecha Retiro</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> dd/mm/aaaa (21/07/2026) y </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t>Novedad</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Arial"/>
+        <family val="2"/>
+      </rPr>
+      <t xml:space="preserve"> es el estado del empleado, en genaral Retirado para esta plantilla</t>
+    </r>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -96,6 +177,13 @@
     <font>
       <b/>
       <sz val="11"/>
+      <name val="Arial"/>
+      <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Arial"/>
       <family val="2"/>
     </font>
@@ -475,6 +563,11 @@
         <v>7</v>
       </c>
     </row>
+    <row r="2" spans="1:7">
+      <c r="A2" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
     <row r="3" spans="1:7">
       <c r="A3" s="2" t="s">
         <v>0</v>
@@ -523,6 +616,11 @@
         <v>10</v>
       </c>
     </row>
+    <row r="2" spans="1:9">
+      <c r="A2" s="1" t="s">
+        <v>12</v>
+      </c>
+    </row>
     <row r="3" spans="1:9">
       <c r="A3" s="3" t="s">
         <v>0</v>

</xml_diff>

<commit_message>
style: ajuste en interfaz grafica
</commit_message>
<xml_diff>
--- a/docs/plantilla-importacion-datos.xlsx
+++ b/docs/plantilla-importacion-datos.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\ASUS\Desktop\coodetrans-gestion\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FDC4CF45-DD6E-4C64-A440-88182D0A84BC}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B688057-ED41-4E8C-82DF-862D2FB72E57}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{B9CF0795-0054-4CD1-8B64-60E772BEE863}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{B9CF0795-0054-4CD1-8B64-60E772BEE863}"/>
   </bookViews>
   <sheets>
     <sheet name="Plantilla para Activos" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="13">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="14">
   <si>
     <t>Codigo</t>
   </si>
@@ -154,6 +154,9 @@
       </rPr>
       <t xml:space="preserve"> es el estado del empleado, en genaral Retirado para esta plantilla</t>
     </r>
+  </si>
+  <si>
+    <t>Genero</t>
   </si>
 </sst>
 </file>
@@ -552,23 +555,26 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E90F8E20-2F8A-46FB-9A93-928A44265DEE}">
-  <dimension ref="A1:G3"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
   <cols>
-    <col min="1" max="16384" width="11.19921875" style="1"/>
+    <col min="1" max="1" width="11.19921875" style="1"/>
+    <col min="2" max="2" width="20.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="9.59765625" style="1" customWidth="1"/>
+    <col min="4" max="16384" width="11.19921875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7">
+    <row r="1" spans="1:8">
       <c r="A1" s="1" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="2" spans="1:7">
+    <row r="2" spans="1:8">
       <c r="A2" s="1" t="s">
         <v>11</v>
       </c>
     </row>
-    <row r="3" spans="1:7">
+    <row r="3" spans="1:8">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
@@ -576,18 +582,21 @@
         <v>1</v>
       </c>
       <c r="C3" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="D3" s="2" t="s">
+      <c r="E3" s="2" t="s">
         <v>3</v>
       </c>
-      <c r="E3" s="2" t="s">
+      <c r="F3" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="G3" s="2" t="s">
         <v>5</v>
       </c>
-      <c r="G3" s="2" t="s">
+      <c r="H3" s="2" t="s">
         <v>6</v>
       </c>
     </row>
@@ -598,30 +607,32 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3DEB0AB-67E2-47F5-A0F7-84CB280836B8}">
-  <dimension ref="A1:I3"/>
+  <dimension ref="A1:J3"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="13.8"/>
   <cols>
     <col min="1" max="1" width="11.19921875" style="1"/>
-    <col min="2" max="2" width="19.8984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.3984375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="11.296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8.69921875" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="8" width="11.19921875" style="1"/>
-    <col min="9" max="9" width="13.19921875" style="1" bestFit="1" customWidth="1"/>
-    <col min="10" max="16384" width="11.19921875" style="1"/>
+    <col min="2" max="2" width="20.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.296875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="10.296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="12" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.69921875" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="9" width="11.19921875" style="1"/>
+    <col min="10" max="10" width="14.09765625" style="1" bestFit="1" customWidth="1"/>
+    <col min="11" max="16384" width="11.19921875" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:10">
       <c r="A1" s="1" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:10">
       <c r="A2" s="1" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:10">
       <c r="A3" s="3" t="s">
         <v>0</v>
       </c>
@@ -629,24 +640,27 @@
         <v>1</v>
       </c>
       <c r="C3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="D3" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="D3" s="3" t="s">
+      <c r="E3" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="E3" s="3" t="s">
+      <c r="F3" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="F3" s="3" t="s">
+      <c r="G3" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="G3" s="3" t="s">
+      <c r="H3" s="3" t="s">
         <v>4</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="I3" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="I3" s="3" t="s">
+      <c r="J3" s="3" t="s">
         <v>6</v>
       </c>
     </row>

</xml_diff>